<commit_message>
Add Source column K to Deduped tab marking CEO-filled rows
Labels all 39 rows where exec names were pulled from CEO Results
sheet as "Pulled from Claude" in the new column K "Source".

https://claude.ai/code/session_01CoqDD8hAVEdkxgHV9GqVZk
</commit_message>
<xml_diff>
--- a/Womens_HRT_updated.xlsx
+++ b/Womens_HRT_updated.xlsx
@@ -14662,7 +14662,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J190"/>
+  <dimension ref="A1:K190"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -14727,6 +14727,11 @@
           <t>Reached Out</t>
         </is>
       </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -14841,6 +14846,11 @@
       <c r="I4" t="n">
         <v>196</v>
       </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Pulled from Claude</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -14906,6 +14916,11 @@
       <c r="I6" t="n">
         <v>22</v>
       </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Pulled from Claude</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -14936,6 +14951,11 @@
       <c r="I7" t="n">
         <v>64</v>
       </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Pulled from Claude</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -15216,6 +15236,11 @@
       <c r="I14" t="n">
         <v>62</v>
       </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Pulled from Claude</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -15246,6 +15271,11 @@
       <c r="I15" t="n">
         <v>64</v>
       </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Pulled from Claude</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -15321,6 +15351,11 @@
       <c r="I17" t="n">
         <v>52</v>
       </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Pulled from Claude</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -15351,6 +15386,11 @@
       <c r="I18" t="n">
         <v>27</v>
       </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Pulled from Claude</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -15381,6 +15421,11 @@
       <c r="I19" t="n">
         <v>20</v>
       </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>Pulled from Claude</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -15411,6 +15456,11 @@
       <c r="I20" t="n">
         <v>22</v>
       </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>Pulled from Claude</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -15441,6 +15491,11 @@
       <c r="I21" t="n">
         <v>42</v>
       </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>Pulled from Claude</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -15471,6 +15526,11 @@
       <c r="I22" t="n">
         <v>26</v>
       </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>Pulled from Claude</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -15501,6 +15561,11 @@
       <c r="I23" t="n">
         <v>261</v>
       </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>Pulled from Claude</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -15531,6 +15596,11 @@
       <c r="I24" t="n">
         <v>25</v>
       </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>Pulled from Claude</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -15561,6 +15631,11 @@
       <c r="I25" t="n">
         <v>30</v>
       </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>Pulled from Claude</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -15591,6 +15666,11 @@
       <c r="I26" t="n">
         <v>94</v>
       </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>Pulled from Claude</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -15621,6 +15701,11 @@
       <c r="I27" t="n">
         <v>92</v>
       </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>Pulled from Claude</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -15651,6 +15736,11 @@
       <c r="I28" t="n">
         <v>32</v>
       </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>Pulled from Claude</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -15681,6 +15771,11 @@
       <c r="I29" t="n">
         <v>40</v>
       </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>Pulled from Claude</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -15711,6 +15806,11 @@
       <c r="I30" t="n">
         <v>53</v>
       </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>Pulled from Claude</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -15781,6 +15881,11 @@
       <c r="I32" t="n">
         <v>21</v>
       </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>Pulled from Claude</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -15811,6 +15916,11 @@
       <c r="I33" t="n">
         <v>21</v>
       </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>Pulled from Claude</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -15841,6 +15951,11 @@
       <c r="I34" t="n">
         <v>28</v>
       </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>Pulled from Claude</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -15866,6 +15981,11 @@
       <c r="I35" t="n">
         <v>34</v>
       </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>Pulled from Claude</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -15896,6 +16016,11 @@
       <c r="I36" t="n">
         <v>82</v>
       </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>Pulled from Claude</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -15926,6 +16051,11 @@
       <c r="I37" t="n">
         <v>75</v>
       </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>Pulled from Claude</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -15956,6 +16086,11 @@
       <c r="I38" t="n">
         <v>237</v>
       </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>Pulled from Claude</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -15986,6 +16121,11 @@
       <c r="I39" t="n">
         <v>495</v>
       </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>Pulled from Claude</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -16016,6 +16156,11 @@
       <c r="I40" t="n">
         <v>316</v>
       </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Pulled from Claude</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -16086,6 +16231,11 @@
       <c r="I42" t="n">
         <v>151</v>
       </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>Pulled from Claude</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -16116,6 +16266,11 @@
       <c r="I43" t="n">
         <v>24</v>
       </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>Pulled from Claude</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -16146,6 +16301,11 @@
       <c r="I44" t="n">
         <v>115</v>
       </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>Pulled from Claude</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -16176,6 +16336,11 @@
       <c r="I45" t="n">
         <v>147</v>
       </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>Pulled from Claude</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -16206,6 +16371,11 @@
       <c r="I46" t="n">
         <v>421</v>
       </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>Pulled from Claude</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -16236,6 +16406,11 @@
       <c r="I47" t="n">
         <v>181</v>
       </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>Pulled from Claude</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -16306,6 +16481,11 @@
       <c r="I49" t="n">
         <v>1498</v>
       </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>Pulled from Claude</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -16336,6 +16516,11 @@
       <c r="I50" t="n">
         <v>78</v>
       </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>Pulled from Claude</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -16406,6 +16591,11 @@
       <c r="I52" t="n">
         <v>730</v>
       </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>Pulled from Claude</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -16436,6 +16626,11 @@
       <c r="I53" t="n">
         <v>284</v>
       </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>Pulled from Claude</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -16465,6 +16660,11 @@
       </c>
       <c r="I54" t="n">
         <v>60</v>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>Pulled from Claude</t>
+        </is>
       </c>
     </row>
     <row r="55">

</xml_diff>

<commit_message>
Add Confidence and Notes columns L and M to Deduped tab
Pulls Confidence and Notes fields from CEO Results sheet for all
39 rows where exec names were sourced from CEO research.

https://claude.ai/code/session_01CoqDD8hAVEdkxgHV9GqVZk
</commit_message>
<xml_diff>
--- a/Womens_HRT_updated.xlsx
+++ b/Womens_HRT_updated.xlsx
@@ -14662,7 +14662,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K190"/>
+  <dimension ref="A1:M190"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -14732,6 +14732,16 @@
           <t>Source</t>
         </is>
       </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Confidence</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -14851,6 +14861,16 @@
           <t>Pulled from Claude</t>
         </is>
       </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>BBB business profile for the Temecula, CA clinic lists Antoinette Jackson-Sekunda as President (business management/principal contact). Corroborated by the company's own JaneApp booking page (bffmedical.janeapp.com) listing her as a provider, and by patient reviews on bffmedical.com referring to 'Dr. Sekunda.' The company's anonymous LinkedIn 'CEO' profile describes a CEO/medical practitioner with a medical degree, consistent with her. Note: Dr. Robert Clendenin, MD is separately listed on bffmedical.com as Medical Director — a distinct clinical-oversight role, not the founder/CEO.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -14921,6 +14941,16 @@
           <t>Pulled from Claude</t>
         </is>
       </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Company's own About page states that in 2023 'Chris' joined with Derrick Adams to launch Mygenics Sarasota, now called Eros Vitality. The About page bio describes Chris as a board-certified Nurse Practitioner who co-founded the clinic. His full surname 'Potter' is confirmed by multiple Google reviews displayed on the same erosvitality.com domain (e.g., 'Chris Potter took the time...'). Derrick Adams is the co-founder/physician partner ('Dr. Adams' / 'Dr. A' in reviews). Both names come directly from the company's own website.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -14956,6 +14986,16 @@
           <t>Pulled from Claude</t>
         </is>
       </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Company's own homepage states the clinic is family-owned with founders Tom and Kitty Houston. Kathryn 'Kitty' Houston is the family nurse practitioner and clinical lead, confirmed via A4M profile listing her at the Roswell, GA address (920 Woodstock Road). Tom Houston is co-founder; if a single name is required, Kathryn (Kitty) Houston is the clinical/medical lead. Both names confirmed for this specific Roswell, GA company.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -15241,6 +15281,16 @@
           <t>Pulled from Claude</t>
         </is>
       </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>The company's own website (primeyouthaesthetics.com) repeatedly states the clinic is 'led by Dr. Yasmine Perdue, DNP, FNP' on the Labs and Skin Care pages, identifying her as the lead provider/medical director for this Pleasanton, CA medspa. No explicit 'CEO' or 'founder' title was found on any source. Note: 'Prime Aesthetics Group' (Co-Founder/CMO Dr. James Chao) is a different, unrelated national plastic surgery network and was excluded. Drew Pagtakhan is the clinic manager, not the leader.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -15276,6 +15326,12 @@
           <t>Pulled from Claude</t>
         </is>
       </c>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>No CEO, founder, or medical director could be confirmed for Restore Youth (restoreyouth.us), the weight loss/wellness/aesthetics clinic in Rancho Cucamonga/Fontana, CA. The company's own site (restoreyouth.us) returned no description, and its social profiles (Instagram @restoreyouth.medical, Facebook, Yelp, Fresha) list no named leader. A LinkedIn result for 'Lorri Manley - CEO at Restore YOUth Med Spa' refers to a DIFFERENT company in Hickory Creek/Lake Dallas, TX (restoreyouthmedspa.com), so it was excluded. A third-party aggregator (TrustAnalytica) mentions a 'Bob NP' as a provider at the Fontana location, but this is only a first name from a low-confidence aggregator and does not clearly identify a CEO/founder/medical director. No reliable name found.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -15356,6 +15412,16 @@
           <t>Pulled from Claude</t>
         </is>
       </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>BBB Business Profile for the correct company (41715 Winchester Rd, Temecula, CA 92590) lists Sharone Utter, Esthetician as Business Management and Principal/Customer Contact. This is corroborated by a testimonial on the company's own product page recommending 'Sharone' for skincare. Title is best described as owner/esthetician rather than CEO/Medical Director; no physician medical director name was identified in the searches. A separate 'Kent Ogden, Marketing Director' was found on a web-design vendor's site, but that is a marketing role, not the founder/CEO. Confidence is Medium because the strongest source is BBB (a business profile clearly identifying this specific company) rather than the company's own About page or a LinkedIn profile.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -15391,6 +15457,16 @@
           <t>Pulled from Claude</t>
         </is>
       </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>The company's own website (webforeveryoung.com, Oakland Park, FL) names Dr. Marc Kaufman MD as the physician leading the medical team alongside 'Elio,' and all medical content on the site is 'medically reviewed by Dr. Marc Kaufman MD, Anti-Aging and Regenerative Medicine Specialist.' Patient testimonials on the site also reference 'Doctor Kaufman.' Note: this is distinct from other similarly named clinics (e.g., Forever Young Medical/Sean Young in Utah, Forever Young Complete Healthcare/Smita Ohri in NJ, 4Ever Young), which are different companies. No separately titled CEO/owner was confirmed on the company's own domain; 'Elio' is mentioned but only by first name with no last name or title found.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -15426,6 +15502,16 @@
           <t>Pulled from Claude</t>
         </is>
       </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>The clinic's own website (evolvelongevitycenter.com) lists 'Van Nguyen M.D.' and all site testimonials reference 'Dr. Van' as the treating physician. A Yelp business listing confirms 'Van Nguyen, MD - Evolve Longevity Center' in Irvine, CA, matching the clinic's address (1820 E Garry Ave, Irvine) and phone (949-486-6006). She appears to be the sole physician/owner of the practice. Exact title (Founder vs. Medical Director) is not explicitly stated on the site, so 'Physician / Medical Director' is the safest characterization.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -15461,6 +15547,12 @@
           <t>Pulled from Claude</t>
         </is>
       </c>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>Company website (balancehrtwell.com) pages returned only general marketing content with no leadership, founder, or medical director names. All named results from searches referred to different, similarly-named companies (Balance Medical in ND, Inner Balance in Boise, Balance My Hormones in UK, Balance Hormone Center in AZ/OK, Balance Financial Wellness, etc.), none of which are this South Florida/Palmetto Bay, FL clinic. No matching LinkedIn or Crunchbase profile for this specific company was found. Cannot confirm a name for the correct company.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -15496,6 +15588,16 @@
           <t>Pulled from Claude</t>
         </is>
       </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>Found on the company's own website (nhvitality.com/the-doctor), where he is identified as 'Dr. Yazan Abdullah, MD MPH, founder and medical director at Newport Health &amp; Vitality.' Confirmed as the right company (Newport Beach, CA hormone/weight-loss clinic) via matching homepage, Yelp listing, and Facebook page. An internist specializing in HRT and medical weight loss.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -15531,6 +15633,16 @@
           <t>Pulled from Claude</t>
         </is>
       </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>Confirmed on the company's own website (healthytransformationmd.com). The company's article explicitly states Dr. Masrour 'founded Healthy Transformation MD,' and multiple pages (homepage, About Us) describe the practice as 'led by Dr. Ojen Masrour,' a board-certified family medicine physician in West Hills, CA. Dr. Lawrence R. Miller is listed as a collaborating physician, and Melat Haile, FNP, is a nurse practitioner, but Dr. Masrour is the founder/lead. Location (West Hills, CA) matches the company's listed address, confirming correct company.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -15566,6 +15678,16 @@
           <t>Pulled from Claude</t>
         </is>
       </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>Found on the company's own About Us page, which states Melissa Kemp is the founder of Georgia Aesthetics &amp; Wellness. Corroborated by her LinkedIn profile (linkedin.com/in/melissa-kemp-60b13958) listing her as Family Nurse Practitioner and aesthetic injector at Georgia Aesthetics and Wellness, and by the clinic email Melissanp@georgiaaesthetics.com on the Locations page. She is also referenced as 'Melissa' in clinic reviews. Location matches (Georgia).</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -15601,6 +15723,16 @@
           <t>Pulled from Claude</t>
         </is>
       </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>Dr. Thom Lobe is consistently identified as the founder and medical director of Regeneveda across multiple sources. The company's own website (regeneveda.com) repeatedly features him as the lead physician overseeing the Chicago and Beverly Hills/LA practice. SlideShare's official Regeneveda account lists him as 'Founder,' Doximity lists him as 'Medical Director, Regeneveda,' and a related clinic site notes he supervises Regeneveda. All sources reference the same Chicago/Beverly Hills locations, confirming this is the correct company.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -15636,6 +15768,16 @@
           <t>Pulled from Claude</t>
         </is>
       </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>Found on the company's own About page at the matching domain (restorativehealthandwellness.org). The page identifies 'our founder Devon Casida, FNP-C' for the medical weight loss clinic in Fresno, CA. The home page testimonials also repeatedly reference 'Devon' as the clinician, confirming this is the correct company and not one of several other unrelated 'Restorative Health &amp; Wellness' practices found in other states (DC, MA, IN, GA, FL).</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -15671,6 +15813,16 @@
           <t>Pulled from Claude</t>
         </is>
       </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>Company's own Providers page states the practice is led by Jennifer Davis, MD, MSCP, who opened San Diego Menopause after being inspired by her own perimenopause journey. Confirmed by her LinkedIn profile (linkedin.com/in/jennifer-davis-md-mscp-990097278) listing San Diego Menopause and matching San Diego location, and corroborated by Yelp and Facebook. While the website does not use the literal word 'founder,' the language 'Before opening San Diego Menopause' and 'led by' clearly identifies her as the founder/lead physician. Note: she is a pediatrics-trained clinician; 'medical director' in her bio refers to a prior UC San Diego role, not necessarily a formal title at this clinic.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -15706,6 +15858,16 @@
           <t>Pulled from Claude</t>
         </is>
       </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>Multiple sources (The Org, LinkedIn profile titled 'Matthew A. Risner - Andrologix Health and Wellness', and RocketReach) identify Matthew (Matt) A. Risner of Jupiter, FL as CEO of Andrologix Health &amp; Wellness. The Org listing is marked 'Unverified', and the LinkedIn profile does not explicitly state his title. The company's own website (andrologix.com / andrologixhealth.com) does not list any leadership team, so the name could not be confirmed on the company domain itself. The RocketReach profile notes he later founded Ultimate Prime Health. Location (Jupiter/West Palm Beach, FL) is consistent across sources, supporting that this is the correct company. Marked Medium because the strongest confirmation comes from third-party profiles rather than the company's own website, and The Org source is unverified.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -15741,6 +15903,16 @@
           <t>Pulled from Claude</t>
         </is>
       </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>The website domain drjosephaiello.com is Dr. Joseph Aiello's own practice (San Diego Center for Integrative Medicine), where the staff is listed as Dr. Joseph Aiello (D.O.), Lisa Marie Rowell, and Elizabeth Farris. A related site (sdintegrativemedicine.com) explicitly titles him 'Medical Director,' and his LinkedIn profile (linkedin.com/in/drjosephaiello) lists drjosephaiello.com as his personal website, confirming the association. NOTE: The name 'San Diego Center For Health' is ambiguous — Yelp/ZoomInfo listings under that exact name refer to a now-closed chiropractic practice (Dr. Llantada / Mindy Mar, DC) at 2333 First Ave, which is a DIFFERENT entity. However, since the provided domain is drjosephaiello.com, the correct associated person is Dr. Joseph Aiello of the San Diego Center for Integrative (Family) Medicine in La Mesa, CA. A Yahoo Local listing also links 'Aiello Joseph P DO' to 'San Diego Center for Health' in La Mesa, supporting this match.</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -15776,6 +15948,16 @@
           <t>Pulled from Claude</t>
         </is>
       </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>Extracted from company name field</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -15811,6 +15993,16 @@
           <t>Pulled from Claude</t>
         </is>
       </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>Company's own website (advmedwell.com) features a first-person About statement attributed to 'Cally Smith APRN, FNP-C' stating she recently opened and formed Advanced Medical Wellness, a concierge medical clinic in Chandler, AZ. The location (Chandler, AZ) matches the business profile, confirming this is the correct company. Title 'Founder' inferred from her statement 'I formed this clinic'; exact CEO/Medical Director title not explicitly stated on site.</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -15886,6 +16078,16 @@
           <t>Pulled from Claude</t>
         </is>
       </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>Company's own About page and Naturopathy page identify Dr. Vahe Melikyan as the founder (N.M.D.) and medical director of Innergy Drips in Scottsdale, AZ. The company website's naturopathy page lists 'Founder &amp; N.M.D.' and includes a personal message signed by Dr. Vahe Melikyan, and the About page states he serves as medical director for Innergy Drips. Dr. Mia Darling is a naturopathic doctor on staff (per her LinkedIn and patient reviews) but is not identified as founder. Found on company-owned domain (innergydrips.com), supporting High confidence.</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -15921,6 +16123,16 @@
           <t>Pulled from Claude</t>
         </is>
       </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>Extracted from company name field</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -15956,6 +16168,12 @@
           <t>Pulled from Claude</t>
         </is>
       </c>
+      <c r="L34" t="inlineStr"/>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>No search results referenced the specific company 'New York HRT' at the domain ny-hrt.com. Results were dominated by unrelated entities sharing the 'HRT' acronym (Hudson River Trading, HRT Solutions HR firm, The HRT Club, Hampton Roads Transit) and various unaffiliated NYC hormone-therapy clinics on different domains (drdecotiis.com, drzilberstein.com, nycintegrative.com, etc.). No content from ny-hrt.com itself or a LinkedIn profile tied to this specific clinic was found, so no leadership name could be reliably confirmed.</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -15986,6 +16204,12 @@
           <t>Pulled from Claude</t>
         </is>
       </c>
+      <c r="L35" t="inlineStr"/>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>No reliable full name for a CEO, founder, or medical director could be confirmed. The clinic (1529 E Interstate 30 #108, Garland, TX 75043) appears to be closed, now referring patients to AD Precision Health. The only personal identifier found is a contact email 'joaquin@tacticalmuscle.com' on the clinic's Facebook page, but a first-name-only email is insufficient to confirm a full name or title. The Bizapedia LLC listing is behind a paywall, and no LinkedIn, Crunchbase, or company About page naming an individual leader was found. Per the no-guessing rule, the name field is left blank.</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -16021,6 +16245,16 @@
           <t>Pulled from Claude</t>
         </is>
       </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>Extracted from company name field</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -16056,6 +16290,16 @@
           <t>Pulled from Claude</t>
         </is>
       </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>Extracted from company name field</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -16091,6 +16335,16 @@
           <t>Pulled from Claude</t>
         </is>
       </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>Confirmed on the company's own website (multiple pages, including the 'Meet Jen' bio page and About page) which identify Jennifer Wright-Bennion, CNM, APRN, as the founder and owner of Luxe Women's Health in Queen Creek, AZ. The gynecology services page explicitly calls her 'our founder and owner.' Corroborated by Manta and ZoomInfo listings for the same Queen Creek, AZ practice. She is a certified nurse-midwife and advanced nurse practitioner who leads the practice; no separate CEO or physician medical director title was found.</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -16126,6 +16380,16 @@
           <t>Pulled from Claude</t>
         </is>
       </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>The company's own website (southshorewc.com) states 'Skilled OB/GYN Larissa Fomitcheva, MD, heads the practice.' Location matches Lindenhurst, NY. Note: the site does not use an explicit 'CEO/founder' title, but it is the only named lead provider and is described as heading the practice. Disambiguated from unrelated similarly-named entities: South Shore Women's Health Care (St. Joseph, MI), South Shore Women's and Children's Hospital (Nigeria, CEO Dr. Olajuwon Alabi), and South Shore Women's Health (Boston, MA).</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -16161,6 +16425,16 @@
           <t>Pulled from Claude</t>
         </is>
       </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>Extracted from company name field</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -16236,6 +16510,16 @@
           <t>Pulled from Claude</t>
         </is>
       </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>Found on company's own About Us page, which lists 'Dr. Peggy Margetson (formerly known as Dr. Roberts), Founder/CEO, Women's Health Expert.' She is a Board-Certified Women's Health Nurse Practitioner in the NY tri-state area (Brooklyn &amp; Deer Park, NY), matching this specific clinic. Earlier 2021 press release on the same domain referred to her as Dr. Peggy Roberts, founder. Name confirmed across the company website and corroborated by Zocdoc provider profile (Dr. Peggy Estime Roberts) for the same Brooklyn/Deer Park locations.</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -16271,6 +16555,16 @@
           <t>Pulled from Claude</t>
         </is>
       </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>The company's own About page confirms the founding provider is 'Kate,' a double board-certified Women's Health Nurse Practitioner and Certified Nurse Midwife who opened her own practice. Patient reviews confirm she founded/opened the practice. However, the company site only provides the first name 'Kate.' A third-party Yahoo Local review page references 'Kathryn Wilson' and 'Katheryn,' but the last name and its spelling could not be confirmed from the company website or a verified LinkedIn profile, so the surname is left blank and confidence is Low. First name 'Kate' is well supported (High confidence) but full name is unconfirmed.</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -16306,6 +16600,16 @@
           <t>Pulled from Claude</t>
         </is>
       </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>Confirmed on the company's own About page (skywomenshealth.com/about), which states Sky Women's Health was 'Founded by Carolyn Moyers, DO, FACOG, MSCP, IF.' The Providers page on the same domain also identifies her as founder. She is a board-certified OB-GYN and Menopause Society Certified Physician based in Fort Worth, TX, matching the company's location. Title 'CEO/Medical Director' is not explicitly stated, but as sole founder and lead physician of this concierge practice she is the clear leader; listed title reflects her role as founder and lead physician.</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -16341,6 +16645,12 @@
           <t>Pulled from Claude</t>
         </is>
       </c>
+      <c r="L45" t="inlineStr"/>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>No reliable CEO, founder, or medical director could be confirmed. Carnegie Women's Health (Manhattan, NYC) was founded in 2019 and is affiliated with Maternal Fetal Medicine Associates. The company's own team page lists multiple physicians (Dr. Sara Kostant, Dr. Aren Gottlieb, Dr. Alison Ho, Dr. Stephanie Lam, Dr. Tamar Goldwaser, Dr. Michael Silverstein) but does NOT designate any individual as founder, CEO, or medical director. No source assigns a specific leadership title to any individual for this clinic, so per the no-guessing rule the name is left blank.</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -16376,6 +16686,16 @@
           <t>Pulled from Claude</t>
         </is>
       </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>Dr. Laquita Martinez is identified across the company's own website (womenblossom.com About and Meet Dr. Martinez pages) as the lead physician of Blossom Women's Health Center in Alpharetta, GA. Her LinkedIn profile (linkedin.com/in/laquita-m-92119185) lists her as Founder of Blossom Women's Health Center, also citing Alpharetta, GA and Morehouse School of Medicine, confirming this is the same person and company. Both High-confidence source types (company domain and personal LinkedIn) agree.</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -16411,6 +16731,16 @@
           <t>Pulled from Claude</t>
         </is>
       </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>Dr. Ann Cha is the founding physician of Women's Health Specialist of North Atlanta in Johns Creek, GA. The practice's own website (achaobgyn.com) and its official Facebook page both identify it as 'Ann Cha, MD OB-GYN located in Johns Creek, GA.' The domain itself (A. Cha OBGYN) reflects her name. Source narrative states she is 'now focused on creating a practice of her own,' confirming founder status. Address (6290 Abbotts Bridge Road, Johns Creek, GA 30097) matches across all sources, confirming this is the correct company. No formal 'CEO' or 'Medical Director' title was published, but as the sole/founding physician she serves in that capacity.</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -16486,6 +16816,16 @@
           <t>Pulled from Claude</t>
         </is>
       </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>Extracted from company name field</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -16521,6 +16861,12 @@
           <t>Pulled from Claude</t>
         </is>
       </c>
+      <c r="L50" t="inlineStr"/>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>The company's official website (thewomenshealthcenter.com) and directory listings (Healthgrades, WebMD, Yelp) confirm this is an OB/GYN group practice in Fountain Valley, CA with multiple physicians (Dr. Lena Nguyen DO, Dr. Linh Nguyen MD, Dr. Beverly Sansone MD, Dr. Elizabeth Tracy MD, etc.), but none of the searches identified a specific person designated as CEO, founder, or medical director. The website's About page does not name a leader, and the only physician bio found (Dr. Lena Nguyen) states she joined the practice in 2015 rather than founded it. No reliable name could be confirmed for a leadership role without guessing.</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -16596,6 +16942,16 @@
           <t>Pulled from Claude</t>
         </is>
       </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>The company's own provider page confirms Dr. Drew Howard, M.D. as a board-certified OB/GYN with the practice. The company About page and multiple sources state the center was founded by 'Dr. Drew and Dr. Kaylar' (the Howards). An Augusta University/MCG article confirms Drew and Kaylar Howard own The Howard Center, the OB/GYN practice they opened in July 2001 in Tifton, GA. Dr. Kaylar G. Howard is the co-founder spouse. Drew Howard listed as primary co-founder; no separate CEO/medical director title was found, but founder/owner is confirmed.</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -16631,6 +16987,12 @@
           <t>Pulled from Claude</t>
         </is>
       </c>
+      <c r="L53" t="inlineStr"/>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>Error: Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfFZ1sVRhCDHZzSXmBA9'}</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -16664,6 +17026,12 @@
       <c r="K54" t="inlineStr">
         <is>
           <t>Pulled from Claude</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr"/>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>Error: Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfFZkaGVzN5kCCiVp82h'}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rebuild HRT sheet with updated CEO data, exec titles, and fixed rows 53-54
- Used updated CEO Results file with corrected data for all rows
- Filled Exec Title column from CEO Results for all matched rows
- Rows 53 & 54 (Women's Health / Nurture) now populated instead of N/A
- Columns K/L/M: Source, Confidence, Notes carried over
- 7 remaining unresolved rows marked N/A with red highlight

https://claude.ai/code/session_01CoqDD8hAVEdkxgHV9GqVZk
</commit_message>
<xml_diff>
--- a/Womens_HRT_updated.xlsx
+++ b/Womens_HRT_updated.xlsx
@@ -14848,6 +14848,11 @@
           <t>1-951-824-6121</t>
         </is>
       </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>President / CEO &amp; Founder</t>
+        </is>
+      </c>
       <c r="H4" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/company/bff-medical-wellness-clinic/</t>
@@ -14933,6 +14938,11 @@
           <t>(941) 777-9142</t>
         </is>
       </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Co-Founder &amp; Nurse Practitioner</t>
+        </is>
+      </c>
       <c r="I6" t="n">
         <v>22</v>
       </c>
@@ -14978,6 +14988,11 @@
           <t>(678) 539-9464</t>
         </is>
       </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Founder &amp; Nurse Practitioner</t>
+        </is>
+      </c>
       <c r="I7" t="n">
         <v>64</v>
       </c>
@@ -15273,6 +15288,11 @@
           <t>1-925-858-4429</t>
         </is>
       </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Lead Nurse Practitioner &amp; Medical Director (DNP, FNP)</t>
+        </is>
+      </c>
       <c r="I14" t="n">
         <v>62</v>
       </c>
@@ -15318,6 +15338,11 @@
           <t>1-909-582-4665</t>
         </is>
       </c>
+      <c r="F15" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="I15" t="n">
         <v>64</v>
       </c>
@@ -15404,6 +15429,11 @@
           <t>1-951-501-1073</t>
         </is>
       </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Owner / Esthetician (Business Management &amp; Principal Contact)</t>
+        </is>
+      </c>
       <c r="I17" t="n">
         <v>52</v>
       </c>
@@ -15449,6 +15479,11 @@
           <t>(954) 361-6067</t>
         </is>
       </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Medical Director / Anti-Aging and Regenerative Medicine Specialist</t>
+        </is>
+      </c>
       <c r="I18" t="n">
         <v>27</v>
       </c>
@@ -15494,6 +15529,11 @@
           <t>(949) 486-6006</t>
         </is>
       </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Physician / Medical Director</t>
+        </is>
+      </c>
       <c r="I19" t="n">
         <v>20</v>
       </c>
@@ -15539,6 +15579,11 @@
           <t>(786) 566-1096</t>
         </is>
       </c>
+      <c r="F20" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="I20" t="n">
         <v>22</v>
       </c>
@@ -15580,6 +15625,11 @@
           <t>1-949-229-5257</t>
         </is>
       </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Founder &amp; Medical Director</t>
+        </is>
+      </c>
       <c r="I21" t="n">
         <v>42</v>
       </c>
@@ -15625,6 +15675,11 @@
           <t>1-818-702-9962</t>
         </is>
       </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Founder &amp; Medical Director (Lead Physician)</t>
+        </is>
+      </c>
       <c r="I22" t="n">
         <v>26</v>
       </c>
@@ -15670,6 +15725,11 @@
           <t>(706) 340-7914</t>
         </is>
       </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Founder &amp; Family Nurse Practitioner</t>
+        </is>
+      </c>
       <c r="I23" t="n">
         <v>261</v>
       </c>
@@ -15715,6 +15775,11 @@
           <t>1-708-979-9148</t>
         </is>
       </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Founder &amp; Medical Director</t>
+        </is>
+      </c>
       <c r="I24" t="n">
         <v>25</v>
       </c>
@@ -15760,6 +15825,11 @@
           <t>(559) 206-7680</t>
         </is>
       </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Founder, FNP-C</t>
+        </is>
+      </c>
       <c r="I25" t="n">
         <v>30</v>
       </c>
@@ -15805,6 +15875,11 @@
           <t>(619) 377-9909</t>
         </is>
       </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Founder &amp; Medical Director (Physician, MD, MSCP)</t>
+        </is>
+      </c>
       <c r="I26" t="n">
         <v>94</v>
       </c>
@@ -15850,6 +15925,11 @@
           <t>(877) 741-6069</t>
         </is>
       </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
       <c r="I27" t="n">
         <v>92</v>
       </c>
@@ -15895,6 +15975,11 @@
           <t>1-619-403-1175</t>
         </is>
       </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Medical Director (Osteopathic Physician, D.O.)</t>
+        </is>
+      </c>
       <c r="I28" t="n">
         <v>32</v>
       </c>
@@ -15940,6 +16025,11 @@
           <t>(912) 335-7825</t>
         </is>
       </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Medical Director</t>
+        </is>
+      </c>
       <c r="I29" t="n">
         <v>40</v>
       </c>
@@ -15985,6 +16075,11 @@
           <t>(480) 542-8204</t>
         </is>
       </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Founder &amp; Nurse Practitioner (APRN, FNP-C)</t>
+        </is>
+      </c>
       <c r="I30" t="n">
         <v>53</v>
       </c>
@@ -16070,6 +16165,11 @@
           <t>(480) 907-5000</t>
         </is>
       </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Founder &amp; Medical Director (N.M.D.)</t>
+        </is>
+      </c>
       <c r="I32" t="n">
         <v>21</v>
       </c>
@@ -16115,6 +16215,11 @@
           <t>(626) 244-3111</t>
         </is>
       </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Medical Director</t>
+        </is>
+      </c>
       <c r="I33" t="n">
         <v>21</v>
       </c>
@@ -16160,6 +16265,11 @@
           <t>(585) 513-6525</t>
         </is>
       </c>
+      <c r="F34" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="I34" t="n">
         <v>28</v>
       </c>
@@ -16196,6 +16306,11 @@
           <t>(469) 461-7044</t>
         </is>
       </c>
+      <c r="F35" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="I35" t="n">
         <v>34</v>
       </c>
@@ -16237,6 +16352,11 @@
           <t>(469) 592-8550</t>
         </is>
       </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Medical Director</t>
+        </is>
+      </c>
       <c r="I36" t="n">
         <v>82</v>
       </c>
@@ -16282,6 +16402,11 @@
           <t>(516) 222-8883</t>
         </is>
       </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Medical Director</t>
+        </is>
+      </c>
       <c r="I37" t="n">
         <v>75</v>
       </c>
@@ -16327,6 +16452,11 @@
           <t>(480) 550-5117</t>
         </is>
       </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Founder &amp; Owner (CNM, APRN)</t>
+        </is>
+      </c>
       <c r="I38" t="n">
         <v>237</v>
       </c>
@@ -16372,6 +16502,11 @@
           <t>1-631-466-5242</t>
         </is>
       </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>OB-GYN / Practice Lead (Medical Director)</t>
+        </is>
+      </c>
       <c r="I39" t="n">
         <v>495</v>
       </c>
@@ -16417,6 +16552,11 @@
           <t>(832) 415-0376</t>
         </is>
       </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Medical Director</t>
+        </is>
+      </c>
       <c r="I40" t="n">
         <v>316</v>
       </c>
@@ -16502,6 +16642,11 @@
           <t>(929) 788-7878</t>
         </is>
       </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Founder &amp; CEO</t>
+        </is>
+      </c>
       <c r="I42" t="n">
         <v>151</v>
       </c>
@@ -16547,6 +16692,11 @@
           <t>(916) 805-5370</t>
         </is>
       </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Founder &amp; Women's Health Nurse Practitioner / Certified Nurse Midwife</t>
+        </is>
+      </c>
       <c r="I43" t="n">
         <v>24</v>
       </c>
@@ -16592,6 +16742,11 @@
           <t>(817) 915-9803</t>
         </is>
       </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Founder &amp; OB-GYN (Medical Director)</t>
+        </is>
+      </c>
       <c r="I44" t="n">
         <v>115</v>
       </c>
@@ -16637,6 +16792,11 @@
           <t>(315) 948-8056</t>
         </is>
       </c>
+      <c r="F45" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="I45" t="n">
         <v>147</v>
       </c>
@@ -16678,6 +16838,11 @@
           <t>(678) 261-7700</t>
         </is>
       </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Founder &amp; Physician (Medical Director)</t>
+        </is>
+      </c>
       <c r="I46" t="n">
         <v>421</v>
       </c>
@@ -16723,6 +16888,11 @@
           <t>(470) 395-4871</t>
         </is>
       </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Founder &amp; OB-GYN (Medical Director)</t>
+        </is>
+      </c>
       <c r="I47" t="n">
         <v>181</v>
       </c>
@@ -16808,6 +16978,11 @@
           <t>(770) 739-1200</t>
         </is>
       </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Medical Director</t>
+        </is>
+      </c>
       <c r="I49" t="n">
         <v>1498</v>
       </c>
@@ -16853,6 +17028,11 @@
           <t>(714) 378-5606</t>
         </is>
       </c>
+      <c r="F50" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="I50" t="n">
         <v>78</v>
       </c>
@@ -16934,6 +17114,11 @@
           <t>(229) 391-3500</t>
         </is>
       </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Co-Founder &amp; OB/GYN (Owner)</t>
+        </is>
+      </c>
       <c r="I52" t="n">
         <v>730</v>
       </c>
@@ -16959,14 +17144,14 @@
           <t>Women's Health (formerly Harmony Center for Women)</t>
         </is>
       </c>
-      <c r="B53" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C53" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Beverly</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Womack</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -16977,6 +17162,11 @@
       <c r="E53" t="inlineStr">
         <is>
           <t>(828) 268-8970</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>OB/GYN Physician &amp; Laboratory Director (no confirmed CEO/Founder/Medical Director title)</t>
         </is>
       </c>
       <c r="I53" t="n">
@@ -16987,10 +17177,14 @@
           <t>Pulled from Claude</t>
         </is>
       </c>
-      <c r="L53" t="inlineStr"/>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>Error: Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfFZ1sVRhCDHZzSXmBA9'}</t>
+          <t>This clinic is owned by Appalachian Regional Healthcare System / UNC Health Appalachian (apprhs.org), not an independently founded practice, and no CEO, founder, or medical director is named on the company's own pages. Dr. Beverly Womack is the most prominent physician tied specifically to this Boone, NC practice: the NPI registry (NPI 1316184807) lists her as 'Laboratory Director' for the practice's CLIA certificate, and a UNC Health Appalachian article notes she joined shortly after Harmony opened in 2008 with 20+ years' experience. However, she is described as a longtime provider, not the founder or designated medical director, so the leadership title cannot be confirmed. Marked Low due to ambiguous/unconfirmed title and health-system ownership.</t>
         </is>
       </c>
     </row>
@@ -17000,14 +17194,14 @@
           <t>Nurture Women's Health and Fertility</t>
         </is>
       </c>
-      <c r="B54" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C54" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Dana</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Ramsey</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -17018,6 +17212,11 @@
       <c r="E54" t="inlineStr">
         <is>
           <t>(831) 515-7078</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Founder &amp; Certified Nurse Midwife (CNM, MSN, RN)</t>
         </is>
       </c>
       <c r="I54" t="n">
@@ -17028,10 +17227,14 @@
           <t>Pulled from Claude</t>
         </is>
       </c>
-      <c r="L54" t="inlineStr"/>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>Error: Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'Your credit balance is too low to access the Anthropic API. Please go to Plans &amp; Billing to upgrade or purchase credits.'}, 'request_id': 'req_011CbfFZkaGVzN5kCCiVp82h'}</t>
+          <t>Confirmed on the company's own website (nurturesantacruz.com) Our Story/Team page, which states Dana Ramsey, CNM, MSN, RN, founded Nurture Women's Health &amp; Fertility after a decade in corporate medicine. The Santa Cruz/Soquel location matches. Note: a similarly named but unrelated 'Nurture Women's Health' in Frisco, TX (co-founded by Drs. Malathi Ellis and Carrie Patterson) also appears in results, but that is a different company; this answer applies to the Santa Cruz practice only.</t>
         </is>
       </c>
     </row>
@@ -21724,6 +21927,26 @@
       <c r="E187" t="inlineStr">
         <is>
           <t>810-955-7949</t>
+        </is>
+      </c>
+      <c r="F187" t="inlineStr">
+        <is>
+          <t>Founder &amp; OB-GYN (Medical Director)</t>
+        </is>
+      </c>
+      <c r="K187" t="inlineStr">
+        <is>
+          <t>Pulled from Claude</t>
+        </is>
+      </c>
+      <c r="L187" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="M187" t="inlineStr">
+        <is>
+          <t>Confirmed on the company's own About page (skywomenshealth.com/about), which states Sky Women's Health was 'Founded by Carolyn Moyers, DO, FACOG, MSCP, IF.' The Providers page on the same domain also identifies her as founder. She is a board-certified OB-GYN and Menopause Society Certified Physician based in Fort Worth, TX, matching the company's location. Title 'CEO/Medical Director' is not explicitly stated, but as sole founder and lead physician of this concierge practice she is the clear leader; listed title reflects her role as founder and lead physician.</t>
         </is>
       </c>
     </row>

</xml_diff>